<commit_message>
Update constraints in FRCoreAdverseEventProfile
Removed constraints for 'detected' and updated 'date' constraint in FRCoreAdverseEventProfile. fd7b1e18d570120da967a694fe223b3da5297a46
</commit_message>
<xml_diff>
--- a/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-adverse-event.xlsx
+++ b/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-adverse-event.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-21T12:27:37+00:00</t>
+    <t>2026-07-30T09:44:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -601,7 +601,7 @@
     <t>AdverseEvent.detected</t>
   </si>
   <si>
-    <t>Date de détection de l'effet indésirable</t>
+    <t>When the event was detected</t>
   </si>
   <si>
     <t>Estimated or actual date the AdverseEvent began, in the opinion of the reporter.</t>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="G17" t="s" s="2">
         <v>86</v>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
         <v>86</v>

</xml_diff>

<commit_message>
feat: ajoute l'extension officielle xver AdverseEvent.occurrence (Period)
Permet de porter la période complète (début + fin) de l'effet
indésirable via le backport R5 officiel occurrence[x] (xver-r5.r4,
http://hl7.org/fhir/5.0/StructureDefinition/extension-AdverseEvent.occurrence),
restreint à Period, en complément de date/resultingCondition.abatementDateTime. d83b3fd0380967378c0565dbd588e068db5d9843
</commit_message>
<xml_diff>
--- a/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-adverse-event.xlsx
+++ b/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-adverse-event.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1890" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2058" uniqueCount="373">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-30T14:33:32+00:00</t>
+    <t>2026-07-30T14:45:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -464,6 +464,100 @@
 </t>
   </si>
   <si>
+    <t>AdverseEvent.extension:occurrence</t>
+  </si>
+  <si>
+    <t>occurrence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://hl7.org/fhir/5.0/StructureDefinition/extension-AdverseEvent.occurrence|0.1.0}
+</t>
+  </si>
+  <si>
+    <t>Période de l'effet indésirable (backport R5 occurrence[x], Period)</t>
+  </si>
+  <si>
+    <t>R5: `AdverseEvent.occurrence[x]` additional types (Period, Timing)</t>
+  </si>
+  <si>
+    <t>Element `AdverseEvent.occurrence[x]` is mapped to FHIR R4 element `AdverseEvent.date` as `SourceIsBroaderThanTarget`.
+The mappings for `AdverseEvent.occurrence[x]` do not cover the following types: Period, Timing.</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension:occurrence.id</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string
+</t>
+  </si>
+  <si>
+    <t>Unique id for inter-element referencing</t>
+  </si>
+  <si>
+    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
+  </si>
+  <si>
+    <t>Element.id</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension:occurrence.extension</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension.extension</t>
+  </si>
+  <si>
+    <t>Extensions are always sliced by (at least) url</t>
+  </si>
+  <si>
+    <t>Element.extension</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension:occurrence.url</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension.url</t>
+  </si>
+  <si>
+    <t>identifies the meaning of the extension</t>
+  </si>
+  <si>
+    <t>Source of the definition for the extension code - a logical name or a URL.</t>
+  </si>
+  <si>
+    <t>The definition may point directly to a computable or human-readable definition of the extensibility codes, or it may be a logical URI as declared in some other specification. The definition SHALL be a URI for the Structure Definition defining the extension.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/5.0/StructureDefinition/extension-AdverseEvent.occurrence</t>
+  </si>
+  <si>
+    <t>Extension.url</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension:occurrence.value[x]</t>
+  </si>
+  <si>
+    <t>AdverseEvent.extension.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period
+</t>
+  </si>
+  <si>
+    <t>When the event occurred</t>
+  </si>
+  <si>
+    <t>The date (and perhaps time) when the adverse event occurred.</t>
+  </si>
+  <si>
+    <t>Extension.value[x]</t>
+  </si>
+  <si>
     <t>AdverseEvent.extension:outcome</t>
   </si>
   <si>
@@ -568,22 +662,6 @@
     <t>AdverseEvent.category.id</t>
   </si>
   <si>
-    <t xml:space="preserve">string
-</t>
-  </si>
-  <si>
-    <t>Unique id for inter-element referencing</t>
-  </si>
-  <si>
-    <t>Unique id for the element within a resource (for internal references). This may be any string value that does not contain spaces.</t>
-  </si>
-  <si>
-    <t>Element.id</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
     <t>AdverseEvent.category.extension</t>
   </si>
   <si>
@@ -591,12 +669,6 @@
   </si>
   <si>
     <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>Extensions are always sliced by (at least) url</t>
-  </si>
-  <si>
-    <t>Element.extension</t>
   </si>
   <si>
     <t>AdverseEvent.category.coding</t>
@@ -831,9 +903,6 @@
   </si>
   <si>
     <t>Date de début de l'effet indésirable</t>
-  </si>
-  <si>
-    <t>The date (and perhaps time) when the adverse event occurred.</t>
   </si>
   <si>
     <t>FiveWs.init</t>
@@ -1417,7 +1486,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AL55"/>
+  <dimension ref="A1:AL60"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="46.7109375" customWidth="true" bestFit="true"/>
@@ -2577,7 +2646,9 @@
       <c r="M11" t="s" s="2">
         <v>148</v>
       </c>
-      <c r="N11" s="2"/>
+      <c r="N11" t="s" s="2">
+        <v>149</v>
+      </c>
       <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
         <v>79</v>
@@ -2649,46 +2720,42 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
-        <v>150</v>
+        <v>79</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I12" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="J12" t="s" s="2">
         <v>79</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>131</v>
+        <v>152</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>152</v>
-      </c>
-      <c r="N12" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="O12" t="s" s="2">
         <v>154</v>
       </c>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
         <v>79</v>
       </c>
@@ -2742,27 +2809,27 @@
         <v>77</v>
       </c>
       <c r="AH12" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI12" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>137</v>
+        <v>79</v>
       </c>
       <c r="AK12" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>129</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2773,7 +2840,7 @@
         <v>77</v>
       </c>
       <c r="G13" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="H13" t="s" s="2">
         <v>79</v>
@@ -2782,23 +2849,19 @@
         <v>79</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>157</v>
+        <v>131</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>158</v>
+        <v>132</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="N13" t="s" s="2">
-        <v>160</v>
-      </c>
-      <c r="O13" t="s" s="2">
-        <v>161</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
         <v>79</v>
       </c>
@@ -2834,31 +2897,31 @@
         <v>79</v>
       </c>
       <c r="AB13" t="s" s="2">
-        <v>79</v>
+        <v>134</v>
       </c>
       <c r="AC13" t="s" s="2">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="AD13" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE13" t="s" s="2">
-        <v>79</v>
+        <v>135</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH13" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI13" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>79</v>
@@ -2869,7 +2932,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B14" t="s" s="2">
         <v>162</v>
@@ -2889,13 +2952,13 @@
         <v>79</v>
       </c>
       <c r="I14" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="J14" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="L14" t="s" s="2">
         <v>163</v>
@@ -2903,14 +2966,16 @@
       <c r="M14" t="s" s="2">
         <v>164</v>
       </c>
-      <c r="N14" s="2"/>
+      <c r="N14" t="s" s="2">
+        <v>165</v>
+      </c>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
         <v>79</v>
       </c>
       <c r="Q14" s="2"/>
       <c r="R14" t="s" s="2">
-        <v>79</v>
+        <v>166</v>
       </c>
       <c r="S14" t="s" s="2">
         <v>79</v>
@@ -2928,32 +2993,32 @@
         <v>79</v>
       </c>
       <c r="X14" t="s" s="2">
-        <v>165</v>
+        <v>79</v>
       </c>
       <c r="Y14" t="s" s="2">
-        <v>166</v>
+        <v>79</v>
       </c>
       <c r="Z14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE14" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF14" t="s" s="2">
         <v>167</v>
       </c>
-      <c r="AA14" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB14" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC14" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD14" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE14" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF14" t="s" s="2">
-        <v>162</v>
-      </c>
       <c r="AG14" t="s" s="2">
         <v>86</v>
       </c>
@@ -2964,18 +3029,18 @@
         <v>79</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>168</v>
+        <v>79</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>79</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>169</v>
@@ -2986,7 +3051,7 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="G15" t="s" s="2">
         <v>86</v>
@@ -2998,7 +3063,7 @@
         <v>79</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K15" t="s" s="2">
         <v>170</v>
@@ -3034,37 +3099,37 @@
         <v>79</v>
       </c>
       <c r="X15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE15" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF15" t="s" s="2">
         <v>173</v>
       </c>
-      <c r="Y15" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="Z15" t="s" s="2">
-        <v>175</v>
-      </c>
-      <c r="AA15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE15" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF15" t="s" s="2">
-        <v>169</v>
-      </c>
       <c r="AG15" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI15" t="s" s="2">
         <v>79</v>
@@ -3073,20 +3138,22 @@
         <v>98</v>
       </c>
       <c r="AK15" t="s" s="2">
-        <v>168</v>
+        <v>79</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>79</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="C16" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="C16" t="s" s="2">
+        <v>175</v>
+      </c>
       <c r="D16" t="s" s="2">
         <v>79</v>
       </c>
@@ -3107,13 +3174,13 @@
         <v>79</v>
       </c>
       <c r="K16" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="L16" t="s" s="2">
         <v>177</v>
       </c>
-      <c r="L16" t="s" s="2">
+      <c r="M16" t="s" s="2">
         <v>178</v>
-      </c>
-      <c r="M16" t="s" s="2">
-        <v>179</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -3164,37 +3231,37 @@
         <v>79</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>180</v>
+        <v>136</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH16" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI16" t="s" s="2">
-        <v>79</v>
+        <v>143</v>
       </c>
       <c r="AJ16" t="s" s="2">
-        <v>79</v>
+        <v>137</v>
       </c>
       <c r="AK16" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>181</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" t="s" s="2">
@@ -3207,7 +3274,7 @@
         <v>79</v>
       </c>
       <c r="I17" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="J17" t="s" s="2">
         <v>79</v>
@@ -3216,15 +3283,17 @@
         <v>131</v>
       </c>
       <c r="L17" t="s" s="2">
+        <v>181</v>
+      </c>
+      <c r="M17" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="N17" t="s" s="2">
         <v>183</v>
       </c>
-      <c r="M17" t="s" s="2">
+      <c r="O17" t="s" s="2">
         <v>184</v>
       </c>
-      <c r="N17" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
         <v>79</v>
       </c>
@@ -3260,19 +3329,19 @@
         <v>79</v>
       </c>
       <c r="AB17" t="s" s="2">
-        <v>134</v>
+        <v>79</v>
       </c>
       <c r="AC17" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>185</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>186</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>77</v>
@@ -3290,15 +3359,15 @@
         <v>79</v>
       </c>
       <c r="AL17" t="s" s="2">
-        <v>181</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -3309,7 +3378,7 @@
         <v>77</v>
       </c>
       <c r="G18" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H18" t="s" s="2">
         <v>79</v>
@@ -3321,19 +3390,19 @@
         <v>87</v>
       </c>
       <c r="K18" t="s" s="2">
+        <v>187</v>
+      </c>
+      <c r="L18" t="s" s="2">
         <v>188</v>
       </c>
-      <c r="L18" t="s" s="2">
+      <c r="M18" t="s" s="2">
         <v>189</v>
       </c>
-      <c r="M18" t="s" s="2">
+      <c r="N18" t="s" s="2">
         <v>190</v>
       </c>
-      <c r="N18" t="s" s="2">
+      <c r="O18" t="s" s="2">
         <v>191</v>
-      </c>
-      <c r="O18" t="s" s="2">
-        <v>192</v>
       </c>
       <c r="P18" t="s" s="2">
         <v>79</v>
@@ -3382,13 +3451,13 @@
         <v>79</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH18" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI18" t="s" s="2">
         <v>79</v>
@@ -3400,15 +3469,15 @@
         <v>79</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>194</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3416,7 +3485,7 @@
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="G19" t="s" s="2">
         <v>86</v>
@@ -3425,19 +3494,19 @@
         <v>79</v>
       </c>
       <c r="I19" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="J19" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>177</v>
+        <v>106</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3464,13 +3533,13 @@
         <v>79</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>79</v>
+        <v>195</v>
       </c>
       <c r="Y19" t="s" s="2">
-        <v>79</v>
+        <v>196</v>
       </c>
       <c r="Z19" t="s" s="2">
-        <v>79</v>
+        <v>197</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>79</v>
@@ -3488,10 +3557,10 @@
         <v>79</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="AG19" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="AH19" t="s" s="2">
         <v>86</v>
@@ -3500,32 +3569,32 @@
         <v>79</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>79</v>
+        <v>198</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>181</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
-        <v>150</v>
+        <v>79</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>79</v>
@@ -3534,20 +3603,18 @@
         <v>79</v>
       </c>
       <c r="J20" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>131</v>
+        <v>200</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="N20" t="s" s="2">
-        <v>153</v>
-      </c>
+        <v>202</v>
+      </c>
+      <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>79</v>
@@ -3572,31 +3639,31 @@
         <v>79</v>
       </c>
       <c r="X20" t="s" s="2">
-        <v>79</v>
+        <v>203</v>
       </c>
       <c r="Y20" t="s" s="2">
-        <v>79</v>
+        <v>204</v>
       </c>
       <c r="Z20" t="s" s="2">
-        <v>79</v>
+        <v>205</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AB20" t="s" s="2">
-        <v>134</v>
+        <v>79</v>
       </c>
       <c r="AC20" t="s" s="2">
-        <v>185</v>
+        <v>79</v>
       </c>
       <c r="AD20" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE20" t="s" s="2">
-        <v>135</v>
+        <v>79</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>77</v>
@@ -3608,21 +3675,21 @@
         <v>79</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>79</v>
+        <v>198</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>181</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3642,23 +3709,19 @@
         <v>79</v>
       </c>
       <c r="J21" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>100</v>
+        <v>152</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>198</v>
+        <v>153</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>199</v>
-      </c>
-      <c r="N21" t="s" s="2">
-        <v>200</v>
-      </c>
-      <c r="O21" t="s" s="2">
-        <v>201</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="N21" s="2"/>
+      <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>79</v>
       </c>
@@ -3667,7 +3730,7 @@
         <v>79</v>
       </c>
       <c r="S21" t="s" s="2">
-        <v>202</v>
+        <v>79</v>
       </c>
       <c r="T21" t="s" s="2">
         <v>79</v>
@@ -3706,7 +3769,7 @@
         <v>79</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>203</v>
+        <v>155</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>77</v>
@@ -3718,32 +3781,32 @@
         <v>79</v>
       </c>
       <c r="AJ21" t="s" s="2">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="AK21" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>204</v>
+        <v>156</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>79</v>
+        <v>180</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G22" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H22" t="s" s="2">
         <v>79</v>
@@ -3752,19 +3815,19 @@
         <v>79</v>
       </c>
       <c r="J22" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>177</v>
+        <v>131</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="N22" t="s" s="2">
-        <v>208</v>
+        <v>183</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" t="s" s="2">
@@ -3802,45 +3865,45 @@
         <v>79</v>
       </c>
       <c r="AB22" t="s" s="2">
-        <v>79</v>
+        <v>134</v>
       </c>
       <c r="AC22" t="s" s="2">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="AD22" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE22" t="s" s="2">
-        <v>79</v>
+        <v>135</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>209</v>
+        <v>160</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH22" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI22" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>210</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3851,7 +3914,7 @@
         <v>77</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>79</v>
@@ -3863,7 +3926,7 @@
         <v>87</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>106</v>
+        <v>211</v>
       </c>
       <c r="L23" t="s" s="2">
         <v>212</v>
@@ -3871,9 +3934,11 @@
       <c r="M23" t="s" s="2">
         <v>213</v>
       </c>
-      <c r="N23" s="2"/>
+      <c r="N23" t="s" s="2">
+        <v>214</v>
+      </c>
       <c r="O23" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P23" t="s" s="2">
         <v>79</v>
@@ -3883,7 +3948,7 @@
         <v>79</v>
       </c>
       <c r="S23" t="s" s="2">
-        <v>215</v>
+        <v>79</v>
       </c>
       <c r="T23" t="s" s="2">
         <v>79</v>
@@ -3928,7 +3993,7 @@
         <v>77</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>79</v>
@@ -3968,21 +4033,19 @@
         <v>79</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>219</v>
+        <v>153</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>220</v>
+        <v>154</v>
       </c>
       <c r="N24" s="2"/>
-      <c r="O24" t="s" s="2">
-        <v>221</v>
-      </c>
+      <c r="O24" s="2"/>
       <c r="P24" t="s" s="2">
         <v>79</v>
       </c>
@@ -4030,7 +4093,7 @@
         <v>79</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>222</v>
+        <v>155</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>77</v>
@@ -4042,32 +4105,32 @@
         <v>79</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="AK24" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>223</v>
+        <v>156</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>79</v>
+        <v>180</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>79</v>
@@ -4076,23 +4139,21 @@
         <v>79</v>
       </c>
       <c r="J25" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>225</v>
+        <v>131</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>226</v>
+        <v>208</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>227</v>
+        <v>209</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>228</v>
-      </c>
-      <c r="O25" t="s" s="2">
-        <v>229</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="O25" s="2"/>
       <c r="P25" t="s" s="2">
         <v>79</v>
       </c>
@@ -4128,45 +4189,45 @@
         <v>79</v>
       </c>
       <c r="AB25" t="s" s="2">
-        <v>79</v>
+        <v>134</v>
       </c>
       <c r="AC25" t="s" s="2">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="AD25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE25" t="s" s="2">
-        <v>79</v>
+        <v>135</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>230</v>
+        <v>160</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="AK25" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>231</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4189,19 +4250,19 @@
         <v>87</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>177</v>
+        <v>100</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>79</v>
@@ -4211,7 +4272,7 @@
         <v>79</v>
       </c>
       <c r="S26" t="s" s="2">
-        <v>79</v>
+        <v>225</v>
       </c>
       <c r="T26" t="s" s="2">
         <v>79</v>
@@ -4250,7 +4311,7 @@
         <v>79</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>77</v>
@@ -4268,15 +4329,15 @@
         <v>79</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>238</v>
+        <v>227</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4287,7 +4348,7 @@
         <v>77</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>79</v>
@@ -4299,15 +4360,17 @@
         <v>87</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>170</v>
+        <v>152</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>241</v>
-      </c>
-      <c r="N27" s="2"/>
+        <v>230</v>
+      </c>
+      <c r="N27" t="s" s="2">
+        <v>231</v>
+      </c>
       <c r="O27" s="2"/>
       <c r="P27" t="s" s="2">
         <v>79</v>
@@ -4332,13 +4395,13 @@
         <v>79</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>242</v>
+        <v>79</v>
       </c>
       <c r="Y27" t="s" s="2">
-        <v>243</v>
+        <v>79</v>
       </c>
       <c r="Z27" t="s" s="2">
-        <v>244</v>
+        <v>79</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>79</v>
@@ -4356,7 +4419,7 @@
         <v>79</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>77</v>
@@ -4371,26 +4434,26 @@
         <v>98</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>245</v>
+        <v>79</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>79</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>247</v>
+        <v>79</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="G28" t="s" s="2">
         <v>86</v>
@@ -4405,19 +4468,17 @@
         <v>87</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>248</v>
+        <v>106</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>249</v>
+        <v>235</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="N28" t="s" s="2">
-        <v>251</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="N28" s="2"/>
       <c r="O28" t="s" s="2">
-        <v>252</v>
+        <v>237</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>79</v>
@@ -4427,7 +4488,7 @@
         <v>79</v>
       </c>
       <c r="S28" t="s" s="2">
-        <v>79</v>
+        <v>238</v>
       </c>
       <c r="T28" t="s" s="2">
         <v>79</v>
@@ -4466,10 +4527,10 @@
         <v>79</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="AG28" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="AH28" t="s" s="2">
         <v>86</v>
@@ -4481,18 +4542,18 @@
         <v>98</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>253</v>
+        <v>79</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>79</v>
+        <v>240</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>254</v>
+        <v>241</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4515,18 +4576,18 @@
         <v>87</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>255</v>
+        <v>152</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="N29" t="s" s="2">
-        <v>258</v>
-      </c>
-      <c r="O29" s="2"/>
+        <v>243</v>
+      </c>
+      <c r="N29" s="2"/>
+      <c r="O29" t="s" s="2">
+        <v>244</v>
+      </c>
       <c r="P29" t="s" s="2">
         <v>79</v>
       </c>
@@ -4574,7 +4635,7 @@
         <v>79</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>77</v>
@@ -4589,18 +4650,18 @@
         <v>98</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>259</v>
+        <v>79</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>79</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>260</v>
+        <v>247</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4623,16 +4684,20 @@
         <v>87</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>261</v>
+        <v>248</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
+        <v>250</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>251</v>
+      </c>
+      <c r="O30" t="s" s="2">
+        <v>252</v>
+      </c>
       <c r="P30" t="s" s="2">
         <v>79</v>
       </c>
@@ -4680,7 +4745,7 @@
         <v>79</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>77</v>
@@ -4695,18 +4760,18 @@
         <v>98</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>264</v>
+        <v>79</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>79</v>
+        <v>254</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4729,16 +4794,20 @@
         <v>87</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>261</v>
+        <v>152</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>267</v>
-      </c>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
+        <v>257</v>
+      </c>
+      <c r="N31" t="s" s="2">
+        <v>258</v>
+      </c>
+      <c r="O31" t="s" s="2">
+        <v>259</v>
+      </c>
       <c r="P31" t="s" s="2">
         <v>79</v>
       </c>
@@ -4786,7 +4855,7 @@
         <v>79</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>77</v>
@@ -4804,15 +4873,15 @@
         <v>79</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>79</v>
+        <v>261</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4823,7 +4892,7 @@
         <v>77</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>79</v>
@@ -4835,17 +4904,15 @@
         <v>87</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>261</v>
+        <v>200</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>270</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>271</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>79</v>
@@ -4870,13 +4937,13 @@
         <v>79</v>
       </c>
       <c r="X32" t="s" s="2">
-        <v>79</v>
+        <v>265</v>
       </c>
       <c r="Y32" t="s" s="2">
-        <v>79</v>
+        <v>266</v>
       </c>
       <c r="Z32" t="s" s="2">
-        <v>79</v>
+        <v>267</v>
       </c>
       <c r="AA32" t="s" s="2">
         <v>79</v>
@@ -4894,7 +4961,7 @@
         <v>79</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>77</v>
@@ -4909,7 +4976,7 @@
         <v>98</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>79</v>
@@ -4917,21 +4984,21 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>79</v>
+        <v>270</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>79</v>
@@ -4943,16 +5010,20 @@
         <v>87</v>
       </c>
       <c r="K33" t="s" s="2">
+        <v>271</v>
+      </c>
+      <c r="L33" t="s" s="2">
+        <v>272</v>
+      </c>
+      <c r="M33" t="s" s="2">
+        <v>273</v>
+      </c>
+      <c r="N33" t="s" s="2">
         <v>274</v>
       </c>
-      <c r="L33" t="s" s="2">
+      <c r="O33" t="s" s="2">
         <v>275</v>
       </c>
-      <c r="M33" t="s" s="2">
-        <v>276</v>
-      </c>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>79</v>
       </c>
@@ -5000,13 +5071,13 @@
         <v>79</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="AG33" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>79</v>
@@ -5015,7 +5086,7 @@
         <v>98</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>79</v>
+        <v>276</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>79</v>
@@ -5057,7 +5128,9 @@
       <c r="M34" t="s" s="2">
         <v>280</v>
       </c>
-      <c r="N34" s="2"/>
+      <c r="N34" t="s" s="2">
+        <v>281</v>
+      </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>79</v>
@@ -5121,7 +5194,7 @@
         <v>98</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>79</v>
+        <v>282</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>79</v>
@@ -5129,10 +5202,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5140,7 +5213,7 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>86</v>
@@ -5155,13 +5228,13 @@
         <v>87</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>170</v>
+        <v>284</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>283</v>
+        <v>172</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5188,11 +5261,13 @@
         <v>79</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>165</v>
-      </c>
-      <c r="Y35" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Y35" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="Z35" t="s" s="2">
-        <v>284</v>
+        <v>79</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>79</v>
@@ -5210,7 +5285,7 @@
         <v>79</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>77</v>
@@ -5225,7 +5300,7 @@
         <v>98</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>79</v>
+        <v>286</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>79</v>
@@ -5233,10 +5308,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5259,13 +5334,13 @@
         <v>87</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>170</v>
+        <v>284</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5292,13 +5367,13 @@
         <v>79</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>165</v>
+        <v>79</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>288</v>
+        <v>79</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>289</v>
+        <v>79</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>79</v>
@@ -5316,7 +5391,7 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>77</v>
@@ -5353,7 +5428,7 @@
         <v>77</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>79</v>
@@ -5365,7 +5440,7 @@
         <v>87</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>170</v>
+        <v>284</v>
       </c>
       <c r="L37" t="s" s="2">
         <v>291</v>
@@ -5373,7 +5448,9 @@
       <c r="M37" t="s" s="2">
         <v>292</v>
       </c>
-      <c r="N37" s="2"/>
+      <c r="N37" t="s" s="2">
+        <v>293</v>
+      </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>79</v>
@@ -5398,13 +5475,13 @@
         <v>79</v>
       </c>
       <c r="X37" t="s" s="2">
-        <v>165</v>
+        <v>79</v>
       </c>
       <c r="Y37" t="s" s="2">
-        <v>293</v>
+        <v>79</v>
       </c>
       <c r="Z37" t="s" s="2">
-        <v>294</v>
+        <v>79</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>79</v>
@@ -5437,7 +5514,7 @@
         <v>98</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>79</v>
+        <v>294</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>79</v>
@@ -5459,7 +5536,7 @@
         <v>77</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>79</v>
@@ -5534,7 +5611,7 @@
         <v>77</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>79</v>
@@ -5543,7 +5620,7 @@
         <v>98</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>299</v>
+        <v>79</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>79</v>
@@ -5551,10 +5628,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5565,7 +5642,7 @@
         <v>77</v>
       </c>
       <c r="G39" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H39" t="s" s="2">
         <v>79</v>
@@ -5577,13 +5654,13 @@
         <v>87</v>
       </c>
       <c r="K39" t="s" s="2">
+        <v>300</v>
+      </c>
+      <c r="L39" t="s" s="2">
         <v>301</v>
       </c>
-      <c r="L39" t="s" s="2">
+      <c r="M39" t="s" s="2">
         <v>302</v>
-      </c>
-      <c r="M39" t="s" s="2">
-        <v>303</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5634,13 +5711,13 @@
         <v>79</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH39" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI39" t="s" s="2">
         <v>79</v>
@@ -5657,10 +5734,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -5671,7 +5748,7 @@
         <v>86</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>79</v>
@@ -5683,13 +5760,13 @@
         <v>87</v>
       </c>
       <c r="K40" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>304</v>
+      </c>
+      <c r="M40" t="s" s="2">
         <v>305</v>
-      </c>
-      <c r="L40" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="M40" t="s" s="2">
-        <v>307</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -5716,13 +5793,11 @@
         <v>79</v>
       </c>
       <c r="X40" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y40" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="Y40" s="2"/>
       <c r="Z40" t="s" s="2">
-        <v>79</v>
+        <v>306</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>79</v>
@@ -5740,13 +5815,13 @@
         <v>79</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>79</v>
@@ -5763,10 +5838,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -5786,16 +5861,16 @@
         <v>79</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>178</v>
+        <v>308</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>179</v>
+        <v>309</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -5822,13 +5897,13 @@
         <v>79</v>
       </c>
       <c r="X41" t="s" s="2">
-        <v>79</v>
+        <v>195</v>
       </c>
       <c r="Y41" t="s" s="2">
-        <v>79</v>
+        <v>310</v>
       </c>
       <c r="Z41" t="s" s="2">
-        <v>79</v>
+        <v>311</v>
       </c>
       <c r="AA41" t="s" s="2">
         <v>79</v>
@@ -5846,7 +5921,7 @@
         <v>79</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>180</v>
+        <v>307</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>77</v>
@@ -5858,32 +5933,32 @@
         <v>79</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="AK41" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>181</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>150</v>
+        <v>79</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>79</v>
@@ -5892,20 +5967,18 @@
         <v>79</v>
       </c>
       <c r="J42" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>131</v>
+        <v>200</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>183</v>
+        <v>313</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>153</v>
-      </c>
+        <v>314</v>
+      </c>
+      <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>79</v>
@@ -5930,13 +6003,13 @@
         <v>79</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>79</v>
+        <v>195</v>
       </c>
       <c r="Y42" t="s" s="2">
-        <v>79</v>
+        <v>315</v>
       </c>
       <c r="Z42" t="s" s="2">
-        <v>79</v>
+        <v>316</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>79</v>
@@ -5954,69 +6027,65 @@
         <v>79</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>186</v>
+        <v>312</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>181</v>
+        <v>79</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>311</v>
+        <v>79</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="J43" t="s" s="2">
         <v>87</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>131</v>
+        <v>318</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>153</v>
-      </c>
-      <c r="O43" t="s" s="2">
-        <v>154</v>
-      </c>
+        <v>320</v>
+      </c>
+      <c r="N43" s="2"/>
+      <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>79</v>
       </c>
@@ -6064,44 +6133,44 @@
         <v>79</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>79</v>
+        <v>321</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>129</v>
+        <v>79</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>316</v>
+        <v>79</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>79</v>
@@ -6113,13 +6182,13 @@
         <v>87</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6170,13 +6239,13 @@
         <v>79</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="AG44" t="s" s="2">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>79</v>
@@ -6193,10 +6262,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6204,10 +6273,10 @@
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>79</v>
@@ -6219,13 +6288,13 @@
         <v>87</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>305</v>
+        <v>327</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6276,7 +6345,7 @@
         <v>79</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>77</v>
@@ -6299,10 +6368,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6325,13 +6394,13 @@
         <v>79</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>178</v>
+        <v>153</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>179</v>
+        <v>154</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -6382,7 +6451,7 @@
         <v>79</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>180</v>
+        <v>155</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>77</v>
@@ -6400,19 +6469,19 @@
         <v>79</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>181</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
@@ -6434,13 +6503,13 @@
         <v>131</v>
       </c>
       <c r="L47" t="s" s="2">
+        <v>208</v>
+      </c>
+      <c r="M47" t="s" s="2">
+        <v>209</v>
+      </c>
+      <c r="N47" t="s" s="2">
         <v>183</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>153</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -6490,7 +6559,7 @@
         <v>79</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>77</v>
@@ -6508,19 +6577,19 @@
         <v>79</v>
       </c>
       <c r="AL47" t="s" s="2">
-        <v>181</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
-        <v>311</v>
+        <v>333</v>
       </c>
       <c r="E48" s="2"/>
       <c r="F48" t="s" s="2">
@@ -6542,16 +6611,16 @@
         <v>131</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>312</v>
+        <v>334</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>313</v>
+        <v>335</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="O48" t="s" s="2">
-        <v>154</v>
+        <v>184</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>79</v>
@@ -6600,7 +6669,7 @@
         <v>79</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>314</v>
+        <v>336</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>77</v>
@@ -6623,14 +6692,14 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
-        <v>79</v>
+        <v>338</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
@@ -6649,13 +6718,13 @@
         <v>87</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>170</v>
+        <v>339</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -6682,11 +6751,13 @@
         <v>79</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>165</v>
-      </c>
-      <c r="Y49" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Y49" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="Z49" t="s" s="2">
-        <v>329</v>
+        <v>79</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>79</v>
@@ -6704,10 +6775,10 @@
         <v>79</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="AG49" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="AH49" t="s" s="2">
         <v>86</v>
@@ -6727,10 +6798,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -6753,13 +6824,13 @@
         <v>87</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>177</v>
+        <v>327</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -6810,13 +6881,13 @@
         <v>79</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH50" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI50" t="s" s="2">
         <v>79</v>
@@ -6833,10 +6904,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -6856,16 +6927,16 @@
         <v>79</v>
       </c>
       <c r="J51" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>334</v>
+        <v>152</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>335</v>
+        <v>153</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>336</v>
+        <v>154</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -6916,7 +6987,7 @@
         <v>79</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>333</v>
+        <v>155</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>77</v>
@@ -6928,32 +6999,32 @@
         <v>79</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>98</v>
+        <v>79</v>
       </c>
       <c r="AK51" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>79</v>
+        <v>156</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>79</v>
+        <v>180</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
         <v>77</v>
       </c>
       <c r="G52" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="H52" t="s" s="2">
         <v>79</v>
@@ -6962,18 +7033,20 @@
         <v>79</v>
       </c>
       <c r="J52" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>338</v>
+        <v>208</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="N52" s="2"/>
+        <v>209</v>
+      </c>
+      <c r="N52" t="s" s="2">
+        <v>183</v>
+      </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
         <v>79</v>
@@ -6998,13 +7071,13 @@
         <v>79</v>
       </c>
       <c r="X52" t="s" s="2">
-        <v>242</v>
+        <v>79</v>
       </c>
       <c r="Y52" t="s" s="2">
-        <v>340</v>
+        <v>79</v>
       </c>
       <c r="Z52" t="s" s="2">
-        <v>341</v>
+        <v>79</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>79</v>
@@ -7022,37 +7095,37 @@
         <v>79</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>337</v>
+        <v>160</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH52" t="s" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="AI52" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ52" t="s" s="2">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="AK52" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL52" t="s" s="2">
-        <v>79</v>
+        <v>156</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>79</v>
+        <v>333</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
@@ -7065,22 +7138,26 @@
         <v>79</v>
       </c>
       <c r="I53" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="J53" t="s" s="2">
         <v>87</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>343</v>
+        <v>131</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>344</v>
-      </c>
-      <c r="N53" s="2"/>
-      <c r="O53" s="2"/>
+        <v>335</v>
+      </c>
+      <c r="N53" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="O53" t="s" s="2">
+        <v>184</v>
+      </c>
       <c r="P53" t="s" s="2">
         <v>79</v>
       </c>
@@ -7128,7 +7205,7 @@
         <v>79</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>77</v>
@@ -7140,21 +7217,21 @@
         <v>79</v>
       </c>
       <c r="AJ53" t="s" s="2">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="AK53" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>79</v>
+        <v>129</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7162,10 +7239,10 @@
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>79</v>
@@ -7177,13 +7254,13 @@
         <v>87</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>346</v>
+        <v>200</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -7210,13 +7287,11 @@
         <v>79</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y54" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>195</v>
+      </c>
+      <c r="Y54" s="2"/>
       <c r="Z54" t="s" s="2">
-        <v>79</v>
+        <v>351</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>79</v>
@@ -7234,13 +7309,13 @@
         <v>79</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI54" t="s" s="2">
         <v>79</v>
@@ -7257,10 +7332,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -7271,7 +7346,7 @@
         <v>77</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="H55" t="s" s="2">
         <v>79</v>
@@ -7283,13 +7358,13 @@
         <v>87</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>349</v>
+        <v>152</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -7340,13 +7415,13 @@
         <v>79</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AH55" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AI55" t="s" s="2">
         <v>79</v>
@@ -7358,6 +7433,536 @@
         <v>79</v>
       </c>
       <c r="AL55" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E56" s="2"/>
+      <c r="F56" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G56" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="H56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J56" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="K56" t="s" s="2">
+        <v>356</v>
+      </c>
+      <c r="L56" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="M56" t="s" s="2">
+        <v>358</v>
+      </c>
+      <c r="N56" s="2"/>
+      <c r="O56" s="2"/>
+      <c r="P56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q56" s="2"/>
+      <c r="R56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF56" t="s" s="2">
+        <v>355</v>
+      </c>
+      <c r="AG56" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH56" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="AI56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ56" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AK56" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL56" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="B57" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E57" s="2"/>
+      <c r="F57" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G57" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="H57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J57" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="K57" t="s" s="2">
+        <v>200</v>
+      </c>
+      <c r="L57" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="M57" t="s" s="2">
+        <v>361</v>
+      </c>
+      <c r="N57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q57" s="2"/>
+      <c r="R57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X57" t="s" s="2">
+        <v>265</v>
+      </c>
+      <c r="Y57" t="s" s="2">
+        <v>362</v>
+      </c>
+      <c r="Z57" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="AA57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF57" t="s" s="2">
+        <v>359</v>
+      </c>
+      <c r="AG57" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH57" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="AI57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ57" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AK57" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL57" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="B58" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E58" s="2"/>
+      <c r="F58" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G58" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J58" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="K58" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="L58" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="M58" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="N58" s="2"/>
+      <c r="O58" s="2"/>
+      <c r="P58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q58" s="2"/>
+      <c r="R58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF58" t="s" s="2">
+        <v>364</v>
+      </c>
+      <c r="AG58" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH58" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ58" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AK58" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL58" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="B59" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E59" s="2"/>
+      <c r="F59" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G59" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J59" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="K59" t="s" s="2">
+        <v>368</v>
+      </c>
+      <c r="L59" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="M59" t="s" s="2">
+        <v>369</v>
+      </c>
+      <c r="N59" s="2"/>
+      <c r="O59" s="2"/>
+      <c r="P59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q59" s="2"/>
+      <c r="R59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF59" t="s" s="2">
+        <v>367</v>
+      </c>
+      <c r="AG59" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH59" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ59" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AK59" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL59" t="s" s="2">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="B60" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="E60" s="2"/>
+      <c r="F60" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G60" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="H60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J60" t="s" s="2">
+        <v>87</v>
+      </c>
+      <c r="K60" t="s" s="2">
+        <v>371</v>
+      </c>
+      <c r="L60" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="M60" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
+      <c r="P60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Q60" s="2"/>
+      <c r="R60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="S60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="T60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="U60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="V60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="W60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="X60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Y60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="Z60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AA60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AB60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AC60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AD60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AE60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AF60" t="s" s="2">
+        <v>370</v>
+      </c>
+      <c r="AG60" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH60" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AJ60" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AK60" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AL60" t="s" s="2">
         <v>79</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restreint suspectEntity.instance à Immunization|Substance|Medication|MedicationAdministration|MedicationStatement
Exclut Procedure et Device (hors périmètre effet indésirable
médicamenteux de ce profil), parmi les types autorisés par la base R4. 29b20dd892447bf1db4d4318354f014435e1e461
</commit_message>
<xml_diff>
--- a/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-adverse-event.xlsx
+++ b/nr-doc-core-adverse-event/ig/StructureDefinition-fr-core-adverse-event.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-30T14:45:27+00:00</t>
+    <t>2026-07-30T14:49:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1072,7 +1072,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(MedicationAdministration|4.0.1)
+    <t xml:space="preserve">Reference(Immunization|4.0.1|Substance|4.0.1|Medication|4.0.1|MedicationAdministration|4.0.1|MedicationStatement|4.0.1)
 </t>
   </si>
   <si>

</xml_diff>